<commit_message>
Add Power BI checks/ingestion pack; use official CF logo & colors
Power BI (CF-Timesheet/powerbi/):
- PowerBI_Model_Notes.md: reverse-engineered the CF_TA Shop Fab model
  (2 pages, 13 tables, 15 measures) from the report definition, plus a
  step-by-step manual rebuild guide (the model binary can't be edited off-Windows)
- PowerQuery_Ingestion.m: paste-ready M for Input - CF Timesheet, Input - Lenel,
  Reference - CF Employees, Reference - CF Activity Types (matches existing naming)
- DAX_Checks.dax: row-level flags + measures for the email's required checks
  (employee names, trades, activity-type mapping, unmatched work orders, and
  booked-hours vs Lenel swipe deviation)

Timesheet template:
- Swapped the placeholder for the official CF logo extracted from the .pbix
- Recolored headers to the CF brand palette (dark green / teal)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EcNn9RiCpngXGpwhkxcwoF
</commit_message>
<xml_diff>
--- a/CF-Timesheet/CF_Timesheet_Template.xlsx
+++ b/CF-Timesheet/CF_Timesheet_Template.xlsx
@@ -45,7 +45,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000B5560"/>
+      <color rgb="00015846"/>
       <sz val="20"/>
     </font>
     <font>
@@ -69,7 +69,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000B5560"/>
+      <color rgb="00015846"/>
       <sz val="10"/>
     </font>
     <font>
@@ -91,7 +91,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B5560"/>
+      <color rgb="00015846"/>
     </font>
     <font>
       <b val="1"/>
@@ -100,12 +100,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B5560"/>
+      <color rgb="00015846"/>
       <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0000848E"/>
+      <color rgb="0000C7B1"/>
       <sz val="12"/>
     </font>
     <font>
@@ -136,7 +136,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B5560"/>
+        <fgColor rgb="00013D30"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,7 +146,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000848E"/>
+        <fgColor rgb="00015846"/>
       </patternFill>
     </fill>
   </fills>
@@ -344,7 +344,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2286000" cy="762000"/>
+    <ext cx="1428750" cy="838200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>[replace logo at B1 with official CF asset]</t>
+          <t>Official CF logo (from CF_TA Shop Fab.pbix)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Style the Wolverine timesheet with the CF look (visual only)
Re-skinned the Wolverine "Timesheet" tab to match the CF template's design
without touching any content:
- CF logo top-left; title -> "CF INDUSTRIES TIMESHEET" in CF green
- CF-green column-header band (white bold) across employee columns and every
  job/PO block; teal totals row; header labels in CF green; gridlines off
- Client sample "Wolverine" -> "CF Industries"
- No values, formulas, dropdowns (13), tables (18), merges, columns/rows, or
  freeze panes changed — verified intact after save

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EcNn9RiCpngXGpwhkxcwoF
</commit_message>
<xml_diff>
--- a/CF-Timesheet/CF_Timesheet_Template.xlsx
+++ b/CF-Timesheet/CF_Timesheet_Template.xlsx
@@ -42,7 +42,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-1009]d/mmm/yy;@"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,8 +115,55 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00015846"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7A77"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B7791F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000A6E5A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2A28"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00015846"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -177,8 +224,23 @@
         <bgColor theme="4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00015846"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000C7B1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A6E5A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -430,12 +492,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -680,6 +756,44 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1098,7 +1212,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1143000" cy="571500"/>
+    <ext cx="1028700" cy="495300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -9289,7 +9403,7 @@
       <c r="EO4" s="21" t="n"/>
       <c r="EP4" s="21" t="n"/>
     </row>
-    <row r="5" ht="18" customFormat="1" customHeight="1" s="17">
+    <row r="5" ht="22" customFormat="1" customHeight="1" s="17">
       <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Blank</t>
@@ -9300,17 +9414,17 @@
           <t>Blank</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>CF INDUSTRIES  —  TA TIMESHEET</t>
-        </is>
-      </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="C5" s="78" t="inlineStr">
+        <is>
+          <t>CF INDUSTRIES TIMESHEET</t>
+        </is>
+      </c>
+      <c r="D5" s="79" t="inlineStr">
         <is>
           <t>Ver. 1.7.1</t>
         </is>
       </c>
-      <c r="H5" s="29" t="inlineStr">
+      <c r="H5" s="80" t="inlineStr">
         <is>
           <t>POPULATE YELLOW HIGHLIGHTED CELLS</t>
         </is>
@@ -9442,12 +9556,12 @@
           <t>Blank</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="81" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="81" t="inlineStr">
         <is>
           <t>Shift</t>
         </is>
@@ -9590,7 +9704,7 @@
           <t>Day</t>
         </is>
       </c>
-      <c r="H7" s="34" t="inlineStr">
+      <c r="H7" s="82" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -9762,7 +9876,7 @@
         <f>IF(C7="","",TEXT(C7,"dddd"))</f>
         <v/>
       </c>
-      <c r="H8" s="34" t="inlineStr">
+      <c r="H8" s="82" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
@@ -9931,7 +10045,7 @@
         </is>
       </c>
       <c r="C9" s="21" t="n"/>
-      <c r="H9" s="34" t="inlineStr">
+      <c r="H9" s="82" t="inlineStr">
         <is>
           <t>Job Desc (not req'd)</t>
         </is>
@@ -10087,7 +10201,7 @@
           <t>Blank</t>
         </is>
       </c>
-      <c r="H10" s="49" t="inlineStr">
+      <c r="H10" s="83" t="inlineStr">
         <is>
           <t>Task Number</t>
         </is>
@@ -10232,7 +10346,7 @@
       <c r="EP10" s="51" t="n"/>
       <c r="EQ10" s="51" t="n"/>
     </row>
-    <row r="11" ht="77.40000000000001" customFormat="1" customHeight="1" s="17">
+    <row r="11" ht="46" customFormat="1" customHeight="1" s="17">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -10243,643 +10357,643 @@
           <t>Blank</t>
         </is>
       </c>
-      <c r="C11" s="45" t="inlineStr">
+      <c r="C11" s="84" t="inlineStr">
         <is>
           <t>Employee Name</t>
         </is>
       </c>
-      <c r="D11" s="45" t="inlineStr">
+      <c r="D11" s="84" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="E11" s="45" t="inlineStr">
+      <c r="E11" s="84" t="inlineStr">
         <is>
           <t>Total Hours</t>
         </is>
       </c>
-      <c r="F11" s="45" t="inlineStr">
+      <c r="F11" s="84" t="inlineStr">
         <is>
           <t>RT Hours</t>
         </is>
       </c>
-      <c r="G11" s="45" t="inlineStr">
+      <c r="G11" s="84" t="inlineStr">
         <is>
           <t>DT Hours</t>
         </is>
       </c>
-      <c r="H11" s="46" t="inlineStr">
+      <c r="H11" s="84" t="inlineStr">
         <is>
           <t>Work Location</t>
         </is>
       </c>
-      <c r="I11" s="46" t="inlineStr">
+      <c r="I11" s="84" t="inlineStr">
         <is>
           <t>Swipe Deviation (if Appr Offsite is used as Hold Up)</t>
         </is>
       </c>
-      <c r="J11" s="46" t="inlineStr">
+      <c r="J11" s="84" t="inlineStr">
         <is>
           <t>Special Rate Considerations (Free Text)</t>
         </is>
       </c>
-      <c r="K11" s="66" t="inlineStr">
+      <c r="K11" s="84" t="inlineStr">
         <is>
           <t>Daily LOA</t>
         </is>
       </c>
-      <c r="L11" s="66" t="inlineStr">
+      <c r="L11" s="84" t="inlineStr">
         <is>
           <t>Which Column?</t>
         </is>
       </c>
-      <c r="M11" s="68" t="inlineStr">
+      <c r="M11" s="84" t="inlineStr">
         <is>
           <t>Meal $$</t>
         </is>
       </c>
-      <c r="N11" s="68" t="inlineStr">
+      <c r="N11" s="84" t="inlineStr">
         <is>
           <t>Which Column?</t>
         </is>
       </c>
-      <c r="O11" s="71" t="inlineStr">
+      <c r="O11" s="84" t="inlineStr">
         <is>
           <t>Meal Order</t>
         </is>
       </c>
-      <c r="P11" s="71" t="inlineStr">
+      <c r="P11" s="84" t="inlineStr">
         <is>
           <t>Which Column?</t>
         </is>
       </c>
-      <c r="Q11" s="47" t="inlineStr">
+      <c r="Q11" s="85" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="R11" s="45" t="inlineStr">
+      <c r="R11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="S11" s="45" t="inlineStr">
+      <c r="S11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="T11" s="45" t="inlineStr">
+      <c r="T11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="U11" s="45" t="inlineStr">
+      <c r="U11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="V11" s="57" t="n"/>
-      <c r="W11" s="46" t="inlineStr">
+      <c r="W11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="X11" s="45" t="inlineStr">
+      <c r="X11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="Y11" s="45" t="inlineStr">
+      <c r="Y11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="Z11" s="45" t="inlineStr">
+      <c r="Z11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="AA11" s="45" t="inlineStr">
+      <c r="AA11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="AB11" s="55" t="n"/>
-      <c r="AC11" s="46" t="inlineStr">
+      <c r="AC11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="AD11" s="45" t="inlineStr">
+      <c r="AD11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="AE11" s="45" t="inlineStr">
+      <c r="AE11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="AF11" s="45" t="inlineStr">
+      <c r="AF11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="AG11" s="45" t="inlineStr">
+      <c r="AG11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="AH11" s="55" t="n"/>
-      <c r="AI11" s="46" t="inlineStr">
+      <c r="AI11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="AJ11" s="45" t="inlineStr">
+      <c r="AJ11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="AK11" s="45" t="inlineStr">
+      <c r="AK11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="AL11" s="45" t="inlineStr">
+      <c r="AL11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="AM11" s="45" t="inlineStr">
+      <c r="AM11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="AN11" s="55" t="n"/>
-      <c r="AO11" s="46" t="inlineStr">
+      <c r="AO11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="AP11" s="45" t="inlineStr">
+      <c r="AP11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="AQ11" s="45" t="inlineStr">
+      <c r="AQ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="AR11" s="45" t="inlineStr">
+      <c r="AR11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="AS11" s="45" t="inlineStr">
+      <c r="AS11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="AT11" s="55" t="n"/>
-      <c r="AU11" s="46" t="inlineStr">
+      <c r="AU11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="AV11" s="45" t="inlineStr">
+      <c r="AV11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="AW11" s="45" t="inlineStr">
+      <c r="AW11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="AX11" s="45" t="inlineStr">
+      <c r="AX11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="AY11" s="45" t="inlineStr">
+      <c r="AY11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="AZ11" s="55" t="n"/>
-      <c r="BA11" s="46" t="inlineStr">
+      <c r="BA11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="BB11" s="45" t="inlineStr">
+      <c r="BB11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="BC11" s="45" t="inlineStr">
+      <c r="BC11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="BD11" s="45" t="inlineStr">
+      <c r="BD11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="BE11" s="45" t="inlineStr">
+      <c r="BE11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="BF11" s="55" t="n"/>
-      <c r="BG11" s="46" t="inlineStr">
+      <c r="BG11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="BH11" s="45" t="inlineStr">
+      <c r="BH11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="BI11" s="45" t="inlineStr">
+      <c r="BI11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="BJ11" s="45" t="inlineStr">
+      <c r="BJ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="BK11" s="45" t="inlineStr">
+      <c r="BK11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="BL11" s="55" t="n"/>
-      <c r="BM11" s="46" t="inlineStr">
+      <c r="BM11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="BN11" s="45" t="inlineStr">
+      <c r="BN11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="BO11" s="45" t="inlineStr">
+      <c r="BO11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="BP11" s="45" t="inlineStr">
+      <c r="BP11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="BQ11" s="45" t="inlineStr">
+      <c r="BQ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="BR11" s="55" t="n"/>
-      <c r="BS11" s="46" t="inlineStr">
+      <c r="BS11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="BT11" s="45" t="inlineStr">
+      <c r="BT11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="BU11" s="45" t="inlineStr">
+      <c r="BU11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="BV11" s="45" t="inlineStr">
+      <c r="BV11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="BW11" s="45" t="inlineStr">
+      <c r="BW11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="BX11" s="55" t="n"/>
-      <c r="BY11" s="46" t="inlineStr">
+      <c r="BY11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="BZ11" s="45" t="inlineStr">
+      <c r="BZ11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="CA11" s="45" t="inlineStr">
+      <c r="CA11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="CB11" s="45" t="inlineStr">
+      <c r="CB11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="CC11" s="45" t="inlineStr">
+      <c r="CC11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="CD11" s="55" t="n"/>
-      <c r="CE11" s="46" t="inlineStr">
+      <c r="CE11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="CF11" s="45" t="inlineStr">
+      <c r="CF11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="CG11" s="45" t="inlineStr">
+      <c r="CG11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="CH11" s="45" t="inlineStr">
+      <c r="CH11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="CI11" s="45" t="inlineStr">
+      <c r="CI11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="CJ11" s="55" t="n"/>
-      <c r="CK11" s="46" t="inlineStr">
+      <c r="CK11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="CL11" s="45" t="inlineStr">
+      <c r="CL11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="CM11" s="45" t="inlineStr">
+      <c r="CM11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="CN11" s="45" t="inlineStr">
+      <c r="CN11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="CO11" s="45" t="inlineStr">
+      <c r="CO11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="CP11" s="55" t="n"/>
-      <c r="CQ11" s="46" t="inlineStr">
+      <c r="CQ11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="CR11" s="45" t="inlineStr">
+      <c r="CR11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="CS11" s="45" t="inlineStr">
+      <c r="CS11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="CT11" s="45" t="inlineStr">
+      <c r="CT11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="CU11" s="45" t="inlineStr">
+      <c r="CU11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="CV11" s="55" t="n"/>
-      <c r="CW11" s="46" t="inlineStr">
+      <c r="CW11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="CX11" s="45" t="inlineStr">
+      <c r="CX11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="CY11" s="45" t="inlineStr">
+      <c r="CY11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="CZ11" s="45" t="inlineStr">
+      <c r="CZ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="DA11" s="45" t="inlineStr">
+      <c r="DA11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="DB11" s="55" t="n"/>
-      <c r="DC11" s="46" t="inlineStr">
+      <c r="DC11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="DD11" s="45" t="inlineStr">
+      <c r="DD11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="DE11" s="45" t="inlineStr">
+      <c r="DE11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="DF11" s="45" t="inlineStr">
+      <c r="DF11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="DG11" s="45" t="inlineStr">
+      <c r="DG11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="DH11" s="55" t="n"/>
-      <c r="DI11" s="46" t="inlineStr">
+      <c r="DI11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="DJ11" s="45" t="inlineStr">
+      <c r="DJ11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="DK11" s="45" t="inlineStr">
+      <c r="DK11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="DL11" s="45" t="inlineStr">
+      <c r="DL11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="DM11" s="45" t="inlineStr">
+      <c r="DM11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="DN11" s="55" t="n"/>
-      <c r="DO11" s="46" t="inlineStr">
+      <c r="DO11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="DP11" s="45" t="inlineStr">
+      <c r="DP11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="DQ11" s="45" t="inlineStr">
+      <c r="DQ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="DR11" s="45" t="inlineStr">
+      <c r="DR11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="DS11" s="45" t="inlineStr">
+      <c r="DS11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="DT11" s="55" t="n"/>
-      <c r="DU11" s="46" t="inlineStr">
+      <c r="DU11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="DV11" s="45" t="inlineStr">
+      <c r="DV11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="DW11" s="45" t="inlineStr">
+      <c r="DW11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="DX11" s="45" t="inlineStr">
+      <c r="DX11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="DY11" s="45" t="inlineStr">
+      <c r="DY11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="DZ11" s="55" t="n"/>
-      <c r="EA11" s="46" t="inlineStr">
+      <c r="EA11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="EB11" s="45" t="inlineStr">
+      <c r="EB11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="EC11" s="45" t="inlineStr">
+      <c r="EC11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="ED11" s="45" t="inlineStr">
+      <c r="ED11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="EE11" s="45" t="inlineStr">
+      <c r="EE11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="EF11" s="55" t="n"/>
-      <c r="EG11" s="46" t="inlineStr">
+      <c r="EG11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="EH11" s="45" t="inlineStr">
+      <c r="EH11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="EI11" s="45" t="inlineStr">
+      <c r="EI11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="EJ11" s="45" t="inlineStr">
+      <c r="EJ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="EK11" s="45" t="inlineStr">
+      <c r="EK11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
       </c>
       <c r="EL11" s="55" t="n"/>
-      <c r="EM11" s="46" t="inlineStr">
+      <c r="EM11" s="84" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="EN11" s="45" t="inlineStr">
+      <c r="EN11" s="84" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="EO11" s="45" t="inlineStr">
+      <c r="EO11" s="84" t="inlineStr">
         <is>
           <t>Hold Up RT</t>
         </is>
       </c>
-      <c r="EP11" s="45" t="inlineStr">
+      <c r="EP11" s="84" t="inlineStr">
         <is>
           <t>Hold Up DT</t>
         </is>
       </c>
-      <c r="EQ11" s="45" t="inlineStr">
+      <c r="EQ11" s="84" t="inlineStr">
         <is>
           <t>Hold Up Type</t>
         </is>
@@ -14235,388 +14349,388 @@
           <t>Blank</t>
         </is>
       </c>
-      <c r="E33" s="25">
+      <c r="E33" s="86">
         <f>SUM(E12:E32)</f>
         <v/>
       </c>
-      <c r="F33" s="25">
+      <c r="F33" s="86">
         <f>SUM(F12:F32)</f>
         <v/>
       </c>
-      <c r="G33" s="25">
+      <c r="G33" s="86">
         <f>SUM(G12:G32)</f>
         <v/>
       </c>
-      <c r="Q33" s="27">
+      <c r="Q33" s="87">
         <f>SUM(Q12:Q32)</f>
         <v/>
       </c>
-      <c r="R33" s="25">
+      <c r="R33" s="86">
         <f>SUM(R12:R32)</f>
         <v/>
       </c>
-      <c r="S33" s="25">
+      <c r="S33" s="86">
         <f>SUM(S12:S32)</f>
         <v/>
       </c>
-      <c r="T33" s="25">
+      <c r="T33" s="86">
         <f>SUM(T12:T32)</f>
         <v/>
       </c>
       <c r="V33" s="60" t="n"/>
-      <c r="W33" s="25">
+      <c r="W33" s="86">
         <f>SUM(W12:W32)</f>
         <v/>
       </c>
-      <c r="X33" s="25">
+      <c r="X33" s="86">
         <f>SUM(X12:X32)</f>
         <v/>
       </c>
-      <c r="Y33" s="25">
+      <c r="Y33" s="86">
         <f>SUM(Y12:Y32)</f>
         <v/>
       </c>
-      <c r="Z33" s="25">
+      <c r="Z33" s="86">
         <f>SUM(Z12:Z32)</f>
         <v/>
       </c>
       <c r="AB33" s="60" t="n"/>
-      <c r="AC33" s="25">
+      <c r="AC33" s="86">
         <f>SUM(AC12:AC32)</f>
         <v/>
       </c>
-      <c r="AD33" s="25">
+      <c r="AD33" s="86">
         <f>SUM(AD12:AD32)</f>
         <v/>
       </c>
-      <c r="AE33" s="25">
+      <c r="AE33" s="86">
         <f>SUM(AE12:AE32)</f>
         <v/>
       </c>
-      <c r="AF33" s="25">
+      <c r="AF33" s="86">
         <f>SUM(AF12:AF32)</f>
         <v/>
       </c>
       <c r="AH33" s="60" t="n"/>
-      <c r="AI33" s="25">
+      <c r="AI33" s="86">
         <f>SUM(AI12:AI32)</f>
         <v/>
       </c>
-      <c r="AJ33" s="25">
+      <c r="AJ33" s="86">
         <f>SUM(AJ12:AJ32)</f>
         <v/>
       </c>
-      <c r="AK33" s="25">
+      <c r="AK33" s="86">
         <f>SUM(AK12:AK32)</f>
         <v/>
       </c>
-      <c r="AL33" s="25">
+      <c r="AL33" s="86">
         <f>SUM(AL12:AL32)</f>
         <v/>
       </c>
       <c r="AN33" s="60" t="n"/>
-      <c r="AO33" s="25">
+      <c r="AO33" s="86">
         <f>SUM(AO12:AO32)</f>
         <v/>
       </c>
-      <c r="AP33" s="25">
+      <c r="AP33" s="86">
         <f>SUM(AP12:AP32)</f>
         <v/>
       </c>
-      <c r="AQ33" s="25">
+      <c r="AQ33" s="86">
         <f>SUM(AQ12:AQ32)</f>
         <v/>
       </c>
-      <c r="AR33" s="25">
+      <c r="AR33" s="86">
         <f>SUM(AR12:AR32)</f>
         <v/>
       </c>
       <c r="AT33" s="60" t="n"/>
-      <c r="AU33" s="25">
+      <c r="AU33" s="86">
         <f>SUM(AU12:AU32)</f>
         <v/>
       </c>
-      <c r="AV33" s="25">
+      <c r="AV33" s="86">
         <f>SUM(AV12:AV32)</f>
         <v/>
       </c>
-      <c r="AW33" s="25">
+      <c r="AW33" s="86">
         <f>SUM(AW12:AW32)</f>
         <v/>
       </c>
-      <c r="AX33" s="25">
+      <c r="AX33" s="86">
         <f>SUM(AX12:AX32)</f>
         <v/>
       </c>
       <c r="AZ33" s="60" t="n"/>
-      <c r="BA33" s="25">
+      <c r="BA33" s="86">
         <f>SUM(BA12:BA32)</f>
         <v/>
       </c>
-      <c r="BB33" s="25">
+      <c r="BB33" s="86">
         <f>SUM(BB12:BB32)</f>
         <v/>
       </c>
-      <c r="BC33" s="25">
+      <c r="BC33" s="86">
         <f>SUM(BC12:BC32)</f>
         <v/>
       </c>
-      <c r="BD33" s="25">
+      <c r="BD33" s="86">
         <f>SUM(BD12:BD32)</f>
         <v/>
       </c>
       <c r="BF33" s="60" t="n"/>
-      <c r="BG33" s="25">
+      <c r="BG33" s="86">
         <f>SUM(BG12:BG32)</f>
         <v/>
       </c>
-      <c r="BH33" s="25">
+      <c r="BH33" s="86">
         <f>SUM(BH12:BH32)</f>
         <v/>
       </c>
-      <c r="BI33" s="25">
+      <c r="BI33" s="86">
         <f>SUM(BI12:BI32)</f>
         <v/>
       </c>
-      <c r="BJ33" s="25">
+      <c r="BJ33" s="86">
         <f>SUM(BJ12:BJ32)</f>
         <v/>
       </c>
       <c r="BL33" s="60" t="n"/>
-      <c r="BM33" s="25">
+      <c r="BM33" s="86">
         <f>SUM(BM12:BM32)</f>
         <v/>
       </c>
-      <c r="BN33" s="25">
+      <c r="BN33" s="86">
         <f>SUM(BN12:BN32)</f>
         <v/>
       </c>
-      <c r="BO33" s="25">
+      <c r="BO33" s="86">
         <f>SUM(BO12:BO32)</f>
         <v/>
       </c>
-      <c r="BP33" s="25">
+      <c r="BP33" s="86">
         <f>SUM(BP12:BP32)</f>
         <v/>
       </c>
       <c r="BR33" s="60" t="n"/>
-      <c r="BS33" s="25">
+      <c r="BS33" s="86">
         <f>SUM(BS12:BS32)</f>
         <v/>
       </c>
-      <c r="BT33" s="25">
+      <c r="BT33" s="86">
         <f>SUM(BT12:BT32)</f>
         <v/>
       </c>
-      <c r="BU33" s="25">
+      <c r="BU33" s="86">
         <f>SUM(BU12:BU32)</f>
         <v/>
       </c>
-      <c r="BV33" s="25">
+      <c r="BV33" s="86">
         <f>SUM(BV12:BV32)</f>
         <v/>
       </c>
       <c r="BX33" s="60" t="n"/>
-      <c r="BY33" s="25">
+      <c r="BY33" s="86">
         <f>SUM(BY12:BY32)</f>
         <v/>
       </c>
-      <c r="BZ33" s="25">
+      <c r="BZ33" s="86">
         <f>SUM(BZ12:BZ32)</f>
         <v/>
       </c>
-      <c r="CA33" s="25">
+      <c r="CA33" s="86">
         <f>SUM(CA12:CA32)</f>
         <v/>
       </c>
-      <c r="CB33" s="25">
+      <c r="CB33" s="86">
         <f>SUM(CB12:CB32)</f>
         <v/>
       </c>
       <c r="CD33" s="60" t="n"/>
-      <c r="CE33" s="25">
+      <c r="CE33" s="86">
         <f>SUM(CE12:CE32)</f>
         <v/>
       </c>
-      <c r="CF33" s="25">
+      <c r="CF33" s="86">
         <f>SUM(CF12:CF32)</f>
         <v/>
       </c>
-      <c r="CG33" s="25">
+      <c r="CG33" s="86">
         <f>SUM(CG12:CG32)</f>
         <v/>
       </c>
-      <c r="CH33" s="25">
+      <c r="CH33" s="86">
         <f>SUM(CH12:CH32)</f>
         <v/>
       </c>
       <c r="CJ33" s="60" t="n"/>
-      <c r="CK33" s="25">
+      <c r="CK33" s="86">
         <f>SUM(CK12:CK32)</f>
         <v/>
       </c>
-      <c r="CL33" s="25">
+      <c r="CL33" s="86">
         <f>SUM(CL12:CL32)</f>
         <v/>
       </c>
-      <c r="CM33" s="25">
+      <c r="CM33" s="86">
         <f>SUM(CM12:CM32)</f>
         <v/>
       </c>
-      <c r="CN33" s="25">
+      <c r="CN33" s="86">
         <f>SUM(CN12:CN32)</f>
         <v/>
       </c>
       <c r="CP33" s="60" t="n"/>
-      <c r="CQ33" s="25">
+      <c r="CQ33" s="86">
         <f>SUM(CQ12:CQ32)</f>
         <v/>
       </c>
-      <c r="CR33" s="25">
+      <c r="CR33" s="86">
         <f>SUM(CR12:CR32)</f>
         <v/>
       </c>
-      <c r="CS33" s="25">
+      <c r="CS33" s="86">
         <f>SUM(CS12:CS32)</f>
         <v/>
       </c>
-      <c r="CT33" s="25">
+      <c r="CT33" s="86">
         <f>SUM(CT12:CT32)</f>
         <v/>
       </c>
       <c r="CV33" s="60" t="n"/>
-      <c r="CW33" s="25">
+      <c r="CW33" s="86">
         <f>SUM(CW12:CW32)</f>
         <v/>
       </c>
-      <c r="CX33" s="25">
+      <c r="CX33" s="86">
         <f>SUM(CX12:CX32)</f>
         <v/>
       </c>
-      <c r="CY33" s="25">
+      <c r="CY33" s="86">
         <f>SUM(CY12:CY32)</f>
         <v/>
       </c>
-      <c r="CZ33" s="25">
+      <c r="CZ33" s="86">
         <f>SUM(CZ12:CZ32)</f>
         <v/>
       </c>
       <c r="DB33" s="60" t="n"/>
-      <c r="DC33" s="25">
+      <c r="DC33" s="86">
         <f>SUM(DC12:DC32)</f>
         <v/>
       </c>
-      <c r="DD33" s="25">
+      <c r="DD33" s="86">
         <f>SUM(DD12:DD32)</f>
         <v/>
       </c>
-      <c r="DE33" s="25">
+      <c r="DE33" s="86">
         <f>SUM(DE12:DE32)</f>
         <v/>
       </c>
-      <c r="DF33" s="25">
+      <c r="DF33" s="86">
         <f>SUM(DF12:DF32)</f>
         <v/>
       </c>
       <c r="DH33" s="60" t="n"/>
-      <c r="DI33" s="25">
+      <c r="DI33" s="86">
         <f>SUM(DI12:DI32)</f>
         <v/>
       </c>
-      <c r="DJ33" s="25">
+      <c r="DJ33" s="86">
         <f>SUM(DJ12:DJ32)</f>
         <v/>
       </c>
-      <c r="DK33" s="25">
+      <c r="DK33" s="86">
         <f>SUM(DK12:DK32)</f>
         <v/>
       </c>
-      <c r="DL33" s="25">
+      <c r="DL33" s="86">
         <f>SUM(DL12:DL32)</f>
         <v/>
       </c>
       <c r="DN33" s="60" t="n"/>
-      <c r="DO33" s="25">
+      <c r="DO33" s="86">
         <f>SUM(DO12:DO32)</f>
         <v/>
       </c>
-      <c r="DP33" s="25">
+      <c r="DP33" s="86">
         <f>SUM(DP12:DP32)</f>
         <v/>
       </c>
-      <c r="DQ33" s="25">
+      <c r="DQ33" s="86">
         <f>SUM(DQ12:DQ32)</f>
         <v/>
       </c>
-      <c r="DR33" s="25">
+      <c r="DR33" s="86">
         <f>SUM(DR12:DR32)</f>
         <v/>
       </c>
       <c r="DT33" s="60" t="n"/>
-      <c r="DU33" s="25">
+      <c r="DU33" s="86">
         <f>SUM(DU12:DU32)</f>
         <v/>
       </c>
-      <c r="DV33" s="25">
+      <c r="DV33" s="86">
         <f>SUM(DV12:DV32)</f>
         <v/>
       </c>
-      <c r="DW33" s="25">
+      <c r="DW33" s="86">
         <f>SUM(DW12:DW32)</f>
         <v/>
       </c>
-      <c r="DX33" s="25">
+      <c r="DX33" s="86">
         <f>SUM(DX12:DX32)</f>
         <v/>
       </c>
       <c r="DZ33" s="60" t="n"/>
-      <c r="EA33" s="25">
+      <c r="EA33" s="86">
         <f>SUM(EA12:EA32)</f>
         <v/>
       </c>
-      <c r="EB33" s="25">
+      <c r="EB33" s="86">
         <f>SUM(EB12:EB32)</f>
         <v/>
       </c>
-      <c r="EC33" s="25">
+      <c r="EC33" s="86">
         <f>SUM(EC12:EC32)</f>
         <v/>
       </c>
-      <c r="ED33" s="25">
+      <c r="ED33" s="86">
         <f>SUM(ED12:ED32)</f>
         <v/>
       </c>
       <c r="EF33" s="60" t="n"/>
-      <c r="EG33" s="25">
+      <c r="EG33" s="86">
         <f>SUM(EG12:EG32)</f>
         <v/>
       </c>
-      <c r="EH33" s="25">
+      <c r="EH33" s="86">
         <f>SUM(EH12:EH32)</f>
         <v/>
       </c>
-      <c r="EI33" s="25">
+      <c r="EI33" s="86">
         <f>SUM(EI12:EI32)</f>
         <v/>
       </c>
-      <c r="EJ33" s="25">
+      <c r="EJ33" s="86">
         <f>SUM(EJ12:EJ32)</f>
         <v/>
       </c>
       <c r="EL33" s="60" t="n"/>
-      <c r="EM33" s="25">
+      <c r="EM33" s="86">
         <f>SUM(EM12:EM32)</f>
         <v/>
       </c>
-      <c r="EN33" s="25">
+      <c r="EN33" s="86">
         <f>SUM(EN12:EN32)</f>
         <v/>
       </c>
-      <c r="EO33" s="25">
+      <c r="EO33" s="86">
         <f>SUM(EO12:EO32)</f>
         <v/>
       </c>
-      <c r="EP33" s="25">
+      <c r="EP33" s="86">
         <f>SUM(EP12:EP32)</f>
         <v/>
       </c>
@@ -14658,7 +14772,7 @@
     <row r="35" ht="21" customFormat="1" customHeight="1" s="15">
       <c r="A35" s="14" t="n"/>
       <c r="B35" s="19" t="n"/>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="88" t="inlineStr">
         <is>
           <t>EQUIPMENT</t>
         </is>
@@ -17589,7 +17703,7 @@
     <row r="53" ht="72" customFormat="1" customHeight="1" s="15">
       <c r="A53" s="14" t="n"/>
       <c r="B53" s="19" t="n"/>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C53" s="89" t="inlineStr">
         <is>
           <t>Description of work accomplished, issues encountered, etc.</t>
         </is>
@@ -17612,220 +17726,220 @@
           <t xml:space="preserve">Job Specific </t>
         </is>
       </c>
-      <c r="R53" s="78" t="n"/>
-      <c r="S53" s="78" t="n"/>
-      <c r="T53" s="78" t="n"/>
-      <c r="U53" s="79" t="n"/>
+      <c r="R53" s="90" t="n"/>
+      <c r="S53" s="90" t="n"/>
+      <c r="T53" s="90" t="n"/>
+      <c r="U53" s="91" t="n"/>
       <c r="V53" s="61" t="n"/>
       <c r="W53" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">Job Specific </t>
         </is>
       </c>
-      <c r="X53" s="78" t="n"/>
-      <c r="Y53" s="78" t="n"/>
-      <c r="Z53" s="78" t="n"/>
-      <c r="AA53" s="79" t="n"/>
+      <c r="X53" s="90" t="n"/>
+      <c r="Y53" s="90" t="n"/>
+      <c r="Z53" s="90" t="n"/>
+      <c r="AA53" s="91" t="n"/>
       <c r="AB53" s="61" t="n"/>
       <c r="AC53" s="76" t="inlineStr">
         <is>
           <t xml:space="preserve">Job Specific </t>
         </is>
       </c>
-      <c r="AD53" s="78" t="n"/>
-      <c r="AE53" s="78" t="n"/>
-      <c r="AF53" s="78" t="n"/>
-      <c r="AG53" s="79" t="n"/>
+      <c r="AD53" s="90" t="n"/>
+      <c r="AE53" s="90" t="n"/>
+      <c r="AF53" s="90" t="n"/>
+      <c r="AG53" s="91" t="n"/>
       <c r="AH53" s="61" t="n"/>
       <c r="AI53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="AJ53" s="78" t="n"/>
-      <c r="AK53" s="78" t="n"/>
-      <c r="AL53" s="78" t="n"/>
-      <c r="AM53" s="79" t="n"/>
+      <c r="AJ53" s="90" t="n"/>
+      <c r="AK53" s="90" t="n"/>
+      <c r="AL53" s="90" t="n"/>
+      <c r="AM53" s="91" t="n"/>
       <c r="AN53" s="61" t="n"/>
       <c r="AO53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="AP53" s="78" t="n"/>
-      <c r="AQ53" s="78" t="n"/>
-      <c r="AR53" s="78" t="n"/>
-      <c r="AS53" s="79" t="n"/>
+      <c r="AP53" s="90" t="n"/>
+      <c r="AQ53" s="90" t="n"/>
+      <c r="AR53" s="90" t="n"/>
+      <c r="AS53" s="91" t="n"/>
       <c r="AT53" s="61" t="n"/>
       <c r="AU53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="AV53" s="78" t="n"/>
-      <c r="AW53" s="78" t="n"/>
-      <c r="AX53" s="78" t="n"/>
-      <c r="AY53" s="79" t="n"/>
+      <c r="AV53" s="90" t="n"/>
+      <c r="AW53" s="90" t="n"/>
+      <c r="AX53" s="90" t="n"/>
+      <c r="AY53" s="91" t="n"/>
       <c r="AZ53" s="61" t="n"/>
       <c r="BA53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="BB53" s="78" t="n"/>
-      <c r="BC53" s="78" t="n"/>
-      <c r="BD53" s="78" t="n"/>
-      <c r="BE53" s="79" t="n"/>
+      <c r="BB53" s="90" t="n"/>
+      <c r="BC53" s="90" t="n"/>
+      <c r="BD53" s="90" t="n"/>
+      <c r="BE53" s="91" t="n"/>
       <c r="BF53" s="61" t="n"/>
       <c r="BG53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="BH53" s="78" t="n"/>
-      <c r="BI53" s="78" t="n"/>
-      <c r="BJ53" s="78" t="n"/>
-      <c r="BK53" s="79" t="n"/>
+      <c r="BH53" s="90" t="n"/>
+      <c r="BI53" s="90" t="n"/>
+      <c r="BJ53" s="90" t="n"/>
+      <c r="BK53" s="91" t="n"/>
       <c r="BL53" s="61" t="n"/>
       <c r="BM53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="BN53" s="78" t="n"/>
-      <c r="BO53" s="78" t="n"/>
-      <c r="BP53" s="78" t="n"/>
-      <c r="BQ53" s="79" t="n"/>
+      <c r="BN53" s="90" t="n"/>
+      <c r="BO53" s="90" t="n"/>
+      <c r="BP53" s="90" t="n"/>
+      <c r="BQ53" s="91" t="n"/>
       <c r="BR53" s="61" t="n"/>
       <c r="BS53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="BT53" s="78" t="n"/>
-      <c r="BU53" s="78" t="n"/>
-      <c r="BV53" s="78" t="n"/>
-      <c r="BW53" s="79" t="n"/>
+      <c r="BT53" s="90" t="n"/>
+      <c r="BU53" s="90" t="n"/>
+      <c r="BV53" s="90" t="n"/>
+      <c r="BW53" s="91" t="n"/>
       <c r="BX53" s="61" t="n"/>
       <c r="BY53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="BZ53" s="78" t="n"/>
-      <c r="CA53" s="78" t="n"/>
-      <c r="CB53" s="78" t="n"/>
-      <c r="CC53" s="79" t="n"/>
+      <c r="BZ53" s="90" t="n"/>
+      <c r="CA53" s="90" t="n"/>
+      <c r="CB53" s="90" t="n"/>
+      <c r="CC53" s="91" t="n"/>
       <c r="CD53" s="61" t="n"/>
       <c r="CE53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="CF53" s="78" t="n"/>
-      <c r="CG53" s="78" t="n"/>
-      <c r="CH53" s="78" t="n"/>
-      <c r="CI53" s="79" t="n"/>
+      <c r="CF53" s="90" t="n"/>
+      <c r="CG53" s="90" t="n"/>
+      <c r="CH53" s="90" t="n"/>
+      <c r="CI53" s="91" t="n"/>
       <c r="CJ53" s="61" t="n"/>
       <c r="CK53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="CL53" s="78" t="n"/>
-      <c r="CM53" s="78" t="n"/>
-      <c r="CN53" s="78" t="n"/>
-      <c r="CO53" s="79" t="n"/>
+      <c r="CL53" s="90" t="n"/>
+      <c r="CM53" s="90" t="n"/>
+      <c r="CN53" s="90" t="n"/>
+      <c r="CO53" s="91" t="n"/>
       <c r="CP53" s="61" t="n"/>
       <c r="CQ53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="CR53" s="78" t="n"/>
-      <c r="CS53" s="78" t="n"/>
-      <c r="CT53" s="78" t="n"/>
-      <c r="CU53" s="79" t="n"/>
+      <c r="CR53" s="90" t="n"/>
+      <c r="CS53" s="90" t="n"/>
+      <c r="CT53" s="90" t="n"/>
+      <c r="CU53" s="91" t="n"/>
       <c r="CV53" s="61" t="n"/>
       <c r="CW53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="CX53" s="78" t="n"/>
-      <c r="CY53" s="78" t="n"/>
-      <c r="CZ53" s="78" t="n"/>
-      <c r="DA53" s="79" t="n"/>
+      <c r="CX53" s="90" t="n"/>
+      <c r="CY53" s="90" t="n"/>
+      <c r="CZ53" s="90" t="n"/>
+      <c r="DA53" s="91" t="n"/>
       <c r="DB53" s="61" t="n"/>
       <c r="DC53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="DD53" s="78" t="n"/>
-      <c r="DE53" s="78" t="n"/>
-      <c r="DF53" s="78" t="n"/>
-      <c r="DG53" s="79" t="n"/>
+      <c r="DD53" s="90" t="n"/>
+      <c r="DE53" s="90" t="n"/>
+      <c r="DF53" s="90" t="n"/>
+      <c r="DG53" s="91" t="n"/>
       <c r="DH53" s="61" t="n"/>
       <c r="DI53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="DJ53" s="78" t="n"/>
-      <c r="DK53" s="78" t="n"/>
-      <c r="DL53" s="78" t="n"/>
-      <c r="DM53" s="79" t="n"/>
+      <c r="DJ53" s="90" t="n"/>
+      <c r="DK53" s="90" t="n"/>
+      <c r="DL53" s="90" t="n"/>
+      <c r="DM53" s="91" t="n"/>
       <c r="DN53" s="61" t="n"/>
       <c r="DO53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="DP53" s="78" t="n"/>
-      <c r="DQ53" s="78" t="n"/>
-      <c r="DR53" s="78" t="n"/>
-      <c r="DS53" s="79" t="n"/>
+      <c r="DP53" s="90" t="n"/>
+      <c r="DQ53" s="90" t="n"/>
+      <c r="DR53" s="90" t="n"/>
+      <c r="DS53" s="91" t="n"/>
       <c r="DT53" s="61" t="n"/>
       <c r="DU53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="DV53" s="78" t="n"/>
-      <c r="DW53" s="78" t="n"/>
-      <c r="DX53" s="78" t="n"/>
-      <c r="DY53" s="79" t="n"/>
+      <c r="DV53" s="90" t="n"/>
+      <c r="DW53" s="90" t="n"/>
+      <c r="DX53" s="90" t="n"/>
+      <c r="DY53" s="91" t="n"/>
       <c r="DZ53" s="61" t="n"/>
       <c r="EA53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="EB53" s="78" t="n"/>
-      <c r="EC53" s="78" t="n"/>
-      <c r="ED53" s="78" t="n"/>
-      <c r="EE53" s="79" t="n"/>
+      <c r="EB53" s="90" t="n"/>
+      <c r="EC53" s="90" t="n"/>
+      <c r="ED53" s="90" t="n"/>
+      <c r="EE53" s="91" t="n"/>
       <c r="EF53" s="61" t="n"/>
       <c r="EG53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="EH53" s="78" t="n"/>
-      <c r="EI53" s="78" t="n"/>
-      <c r="EJ53" s="78" t="n"/>
-      <c r="EK53" s="79" t="n"/>
+      <c r="EH53" s="90" t="n"/>
+      <c r="EI53" s="90" t="n"/>
+      <c r="EJ53" s="90" t="n"/>
+      <c r="EK53" s="91" t="n"/>
       <c r="EL53" s="61" t="n"/>
       <c r="EM53" s="76" t="inlineStr">
         <is>
           <t>Job Specific</t>
         </is>
       </c>
-      <c r="EN53" s="78" t="n"/>
-      <c r="EO53" s="78" t="n"/>
-      <c r="EP53" s="78" t="n"/>
-      <c r="EQ53" s="79" t="n"/>
+      <c r="EN53" s="90" t="n"/>
+      <c r="EO53" s="90" t="n"/>
+      <c r="EP53" s="90" t="n"/>
+      <c r="EQ53" s="91" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>